<commit_message>
sync: update product data files from Google Sheets
</commit_message>
<xml_diff>
--- a/سفارش 1405.xlsx
+++ b/سفارش 1405.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A123DEF-2D64-4114-B1E3-8781ABCEEABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87797D2C-FE6F-46CA-BEDC-2696B88BD457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1017,7 +1017,7 @@
         <v>1522600</v>
       </c>
       <c r="K2" s="1">
-        <v>1914400</v>
+        <v>1900000</v>
       </c>
       <c r="L2" s="1">
         <f t="shared" ref="L2:L7" si="4">SUM(M2:AZ2)</f>

</xml_diff>